<commit_message>
Fájlstruktúra, navbar, footer, bootstrap implementálás, template létrehozása
létrehoztam minden html fájlt, képek, css, scriptek strukturálása, navbar és footer elkészítése, betölthető minden oldalon. Template mappában található az alap oldalszerkezet, csak ki kell másolni és be kell illeszteni minden oldalra kiindulásként.
</commit_message>
<xml_diff>
--- a/dokumentumok/munkaido_naplo.xlsx
+++ b/dokumentumok/munkaido_naplo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sedla\Desktop\napfenysziget weboldal\dokumentumok\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sedla\Desktop\napfenysziget-alapitvany\dokumentumok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{593EDF5B-4AA2-4D09-A377-16442BFCA784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D76515-7B0D-4D45-8EC6-9022D8CD4128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>elkezdtem</t>
   </si>
@@ -46,6 +46,12 @@
   </si>
   <si>
     <t>a global-data.js scriptet csinaltam meg, amibe az alapitvany fontos adatait tarolom (pl nev,adoszam stb). HTML elemkent felhasznalhatoak</t>
+  </si>
+  <si>
+    <t>fájlstruktúra létrehozása, bootstrap importálása, html és css a bootstraphez igazítása</t>
+  </si>
+  <si>
+    <t>navbar és footer elkészítése és globalizálása (egy helyen megírom, minden oldalon betöltöm a nav-footer.js scripttel), template létrehozása</t>
   </si>
 </sst>
 </file>
@@ -99,7 +105,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normál" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -377,16 +383,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="126.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="158" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -400,7 +406,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>46152</v>
       </c>
@@ -414,7 +420,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>46164</v>
       </c>
@@ -428,7 +434,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>46174</v>
       </c>
@@ -440,6 +446,34 @@
       </c>
       <c r="D4" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>46180</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>46180</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0.57638888888888884</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
impresszum és oldaltérkép elkészitése, bugfix, global-data.js kiegészitése
</commit_message>
<xml_diff>
--- a/dokumentumok/munkaido_naplo.xlsx
+++ b/dokumentumok/munkaido_naplo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sedla\Desktop\napfenysziget-alapitvany\dokumentumok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D76515-7B0D-4D45-8EC6-9022D8CD4128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7B7FD88-71DD-4C53-ABB3-F5D1488585BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>elkezdtem</t>
   </si>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t>navbar és footer elkészítése és globalizálása (egy helyen megírom, minden oldalon betöltöm a nav-footer.js scripttel), template létrehozása</t>
+  </si>
+  <si>
+    <t>Tovabbi stilus modositasok, impresszum oldal megfelelo adatainak kutatasa, oldalterkep es impresszum oldal elkeszitese, "alapitvany-domain" custom HTML element hozzadasa a global-data.js fajlhoz</t>
   </si>
 </sst>
 </file>
@@ -105,7 +108,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normál" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -383,16 +386,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="14.5546875" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="158" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="181" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -406,7 +409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>46152</v>
       </c>
@@ -420,7 +423,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>46164</v>
       </c>
@@ -434,7 +437,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>46174</v>
       </c>
@@ -448,7 +451,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>46180</v>
       </c>
@@ -462,7 +465,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>46180</v>
       </c>
@@ -474,6 +477,20 @@
       </c>
       <c r="D6" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>46189</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fooldal elkeszitese a megkuldott szoveg alapjan, az elkuldott szovegeket elkezdtem berakni a HTML fajlokba.
</commit_message>
<xml_diff>
--- a/dokumentumok/munkaido_naplo.xlsx
+++ b/dokumentumok/munkaido_naplo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sedla\Desktop\napfenysziget-alapitvany\dokumentumok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7B7FD88-71DD-4C53-ABB3-F5D1488585BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{255A2BA3-14D8-45D6-8183-7605010A5262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>elkezdtem</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>Tovabbi stilus modositasok, impresszum oldal megfelelo adatainak kutatasa, oldalterkep es impresszum oldal elkeszitese, "alapitvany-domain" custom HTML element hozzadasa a global-data.js fajlhoz</t>
+  </si>
+  <si>
+    <t>Fooldal elkeszitese a megkuldott szoveg alapjan, az elkuldott szovegeket elkezdtem berakni a HTML fajlokba.</t>
   </si>
 </sst>
 </file>
@@ -99,16 +102,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normál" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -386,16 +398,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="181" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -409,7 +421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>46152</v>
       </c>
@@ -419,11 +431,11 @@
       <c r="C2" s="2">
         <v>0.75694444444444442</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>46164</v>
       </c>
@@ -433,11 +445,11 @@
       <c r="C3" s="2">
         <v>0.53125</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>46174</v>
       </c>
@@ -447,11 +459,11 @@
       <c r="C4" s="2">
         <v>0.69444444444444442</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>46180</v>
       </c>
@@ -461,11 +473,11 @@
       <c r="C5" s="2">
         <v>0.55555555555555558</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>46180</v>
       </c>
@@ -475,11 +487,11 @@
       <c r="C6" s="2">
         <v>0.63541666666666663</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>46189</v>
       </c>
@@ -489,11 +501,51 @@
       <c r="C7" s="2">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="4" t="s">
         <v>9</v>
       </c>
     </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>46191</v>
+      </c>
+      <c r="B8" s="2">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0.3611111111111111</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>46191</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0.4201388888888889</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>46191</v>
+      </c>
+      <c r="B10" s="6">
+        <v>0.50347222222222221</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B11" s="2"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D8:D9"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
tamogatas, rolunk, kuldetesunk, celjaink szovegenek beillesztese, index stilus modositasa, tamogatas css elkeszitese
</commit_message>
<xml_diff>
--- a/dokumentumok/munkaido_naplo.xlsx
+++ b/dokumentumok/munkaido_naplo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sedla\Desktop\napfenysziget-alapitvany\dokumentumok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{255A2BA3-14D8-45D6-8183-7605010A5262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC60632C-DDDF-4867-ABA3-6133763369C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>elkezdtem</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>Fooldal elkeszitese a megkuldott szoveg alapjan, az elkuldott szovegeket elkezdtem berakni a HTML fajlokba.</t>
+  </si>
+  <si>
+    <t>tamogatas, rolunk, kuldetesunk, celjaink szovegenek beillesztese, index stilus modositasa, tamogatas css elkeszitese</t>
   </si>
 </sst>
 </file>
@@ -112,10 +115,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -515,7 +518,7 @@
       <c r="C8" s="2">
         <v>0.3611111111111111</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>10</v>
       </c>
     </row>
@@ -529,14 +532,20 @@
       <c r="C9" s="2">
         <v>0.45833333333333331</v>
       </c>
-      <c r="D9" s="5"/>
+      <c r="D9" s="6"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>46191</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="5">
         <v>0.50347222222222221</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.53819444444444442</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
képek leszedése, beillesztés, oldaltérkép módosítása, kapcsolat oldal elkészítése
Egy képet használtam fel a rólunk oldalon, többi majd a tevékenységek/hírek és tevékenységek galéria oldalon lesz felhasználva. Az oldalterkep.html oldalról kiszedtem az online adományozás és adó 1% linket, mert feleslegesnek tartom a jelenlegi koncepció szerint.
</commit_message>
<xml_diff>
--- a/dokumentumok/munkaido_naplo.xlsx
+++ b/dokumentumok/munkaido_naplo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sedla\Desktop\napfenysziget-alapitvany\dokumentumok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC60632C-DDDF-4867-ABA3-6133763369C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199A2E9E-B408-46D2-82CD-D5E63DFE85B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>elkezdtem</t>
   </si>
@@ -61,6 +61,12 @@
   </si>
   <si>
     <t>tamogatas, rolunk, kuldetesunk, celjaink szovegenek beillesztese, index stilus modositasa, tamogatas css elkeszitese</t>
+  </si>
+  <si>
+    <t>Kepek leszedese, beillesztése a rolunk oldalra</t>
+  </si>
+  <si>
+    <t>kapcsolat oldal elkészítése</t>
   </si>
 </sst>
 </file>
@@ -401,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -549,7 +555,32 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="2"/>
+      <c r="A11" s="1">
+        <v>46193</v>
+      </c>
+      <c r="B11" s="2">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>46218</v>
+      </c>
+      <c r="B12" s="2">
+        <v>0.61111111111111116</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.64236111111111116</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Hirek oldal, programunk oldal, stilus elkeszites, kodolas veglegesitese, dokumentacio befejezese (attekintest meg igenyel), 2 todo kiirasa, commit githubra
dokumentaciot at kell nezni meg, es a 2 todo-t el kell vegezni! A kepek amik a github szerint torlesre kerultek, azok csak atnevezesre kerultek! valamint atraktam a nem hasznalt oldalakat egy archive nevu mappaba.
</commit_message>
<xml_diff>
--- a/dokumentumok/munkaido_naplo.xlsx
+++ b/dokumentumok/munkaido_naplo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sedla\Desktop\napfenysziget-alapitvany\dokumentumok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199A2E9E-B408-46D2-82CD-D5E63DFE85B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38709F5-D167-4208-A345-C534ACB3950A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>elkezdtem</t>
   </si>
@@ -67,6 +67,12 @@
   </si>
   <si>
     <t>kapcsolat oldal elkészítése</t>
+  </si>
+  <si>
+    <t>Hirek oldal, programunk oldal, stilus elkeszites, kodolas veglegesitese, dokumentalas (nem fejeztem be, tancom van)</t>
+  </si>
+  <si>
+    <t>dokumentacio befejezese (attekintest meg igenyel), 2 todo kiirasa, commit githubra</t>
   </si>
 </sst>
 </file>
@@ -129,7 +135,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normál" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -407,16 +413,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="14.5546875" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="181" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -430,7 +436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>46152</v>
       </c>
@@ -444,7 +450,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>46164</v>
       </c>
@@ -458,7 +464,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>46174</v>
       </c>
@@ -472,7 +478,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>46180</v>
       </c>
@@ -486,7 +492,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>46180</v>
       </c>
@@ -500,7 +506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>46189</v>
       </c>
@@ -514,7 +520,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>46191</v>
       </c>
@@ -528,7 +534,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>46191</v>
       </c>
@@ -540,7 +546,7 @@
       </c>
       <c r="D9" s="6"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>46191</v>
       </c>
@@ -554,7 +560,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>46193</v>
       </c>
@@ -568,7 +574,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>46218</v>
       </c>
@@ -580,6 +586,34 @@
       </c>
       <c r="D12" s="4" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>46265</v>
+      </c>
+      <c r="B13" s="2">
+        <v>0.59375</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0.78125</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B14" s="2">
+        <v>0.4375</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0.4513888888888889</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>